<commit_message>
feat(calculators): implement method 2 for 3.5 swine methane
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.5-swine-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.5-swine-enteric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{1B232D4B-2524-5A49-BDBA-FB4ED37B618E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{F10DCDEC-1430-924E-8BBA-1FB3E909157D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51220" yWindow="18380" windowWidth="28800" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
   <si>
     <t>(Ij * 18.6 * 0.007) / F</t>
   </si>
@@ -165,28 +165,13 @@
     <t>Nitrogen waste</t>
   </si>
   <si>
-    <t>Outdoor (Dry lot) </t>
-  </si>
-  <si>
-    <t>Deep litter </t>
-  </si>
-  <si>
-    <t>Stockpile (Solid storage) </t>
-  </si>
-  <si>
-    <t>Effluent pond (Uncovered anaerobic lagoon) </t>
-  </si>
-  <si>
-    <t>Anaerobic digester / Covered lagoon </t>
-  </si>
-  <si>
-    <t>Short HRT tank storage &lt; 1 month (pit storage) </t>
-  </si>
-  <si>
-    <t>MMSm</t>
-  </si>
-  <si>
     <t>MJ/kg CH4</t>
+  </si>
+  <si>
+    <t>Mostly zeros</t>
+  </si>
+  <si>
+    <t>Method 2 - Custom Ij</t>
   </si>
 </sst>
 </file>
@@ -583,7 +568,7 @@
   <dimension ref="A2:S34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
     <col min="16" max="16" width="12.5" customWidth="1"/>
   </cols>
@@ -622,7 +607,7 @@
         <v>55.22</v>
       </c>
       <c r="R3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -918,14 +903,9 @@
         <v>798.31792828685263</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="P15" t="s">
-        <v>49</v>
-      </c>
-    </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
         <v>34</v>
@@ -956,12 +936,8 @@
         <f>SUM(I16:I20)*10^-3</f>
         <v>0.88701992031872523</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
@@ -989,12 +965,8 @@
         <f t="shared" ref="I17:I19" si="7">F17*G17*H17</f>
         <v>0</v>
       </c>
-      <c r="P17" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q17" s="3">
-        <v>0.125</v>
-      </c>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
@@ -1022,12 +994,8 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="P18" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q18" s="3">
-        <v>0.2</v>
-      </c>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
@@ -1055,142 +1023,138 @@
         <f t="shared" si="7"/>
         <v>887.01992031872521</v>
       </c>
-      <c r="P19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q19" s="3">
-        <v>0.55000000000000004</v>
-      </c>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="P20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q20" s="3">
-        <v>0</v>
-      </c>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="P21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>0.25</v>
-      </c>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
       </c>
-      <c r="D31">
-        <f>$Q$10</f>
-        <v>2.62</v>
+      <c r="C31" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="D31" s="2">
+        <v>2.5</v>
       </c>
       <c r="E31">
         <f>$Q$3</f>
         <v>55.22</v>
       </c>
       <c r="F31">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="G31">
         <f>(D31 * 18.6 * 0.007) / E31</f>
-        <v>6.1775443679826158E-3</v>
+        <v>5.8946034045635641E-3</v>
       </c>
       <c r="H31">
         <v>365</v>
       </c>
       <c r="I31">
         <f>F31*G31*H31</f>
-        <v>1803.8429554509239</v>
+        <v>1075.7651213328504</v>
       </c>
       <c r="J31">
-        <f>SUM(I21:I25)*10^-3</f>
-        <v>0</v>
+        <f>SUM(I31:I35)*10^-3</f>
+        <v>4.1480229844259329</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>35</v>
       </c>
-      <c r="D32">
-        <f>$Q$11</f>
-        <v>2.2999999999999998</v>
+      <c r="C32" s="2">
+        <v>2.1</v>
+      </c>
+      <c r="D32" s="2">
+        <v>2.1</v>
       </c>
       <c r="E32">
         <f t="shared" ref="E32:E34" si="8">$Q$3</f>
         <v>55.22</v>
       </c>
       <c r="F32">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="G32">
         <f t="shared" ref="G32:G34" si="9">(D32 * 18.6 * 0.007) / E32</f>
-        <v>5.4230351321984793E-3</v>
+        <v>4.9514668598333936E-3</v>
       </c>
       <c r="H32">
         <v>365</v>
       </c>
       <c r="I32">
         <f t="shared" ref="I32:I34" si="10">F32*G32*H32</f>
-        <v>2375.2893879029339</v>
+        <v>1988.0139442231077</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>36</v>
       </c>
-      <c r="D33">
-        <f>$Q$12</f>
-        <v>2.5</v>
+      <c r="C33" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="D33" s="2">
+        <v>2.6</v>
       </c>
       <c r="E33">
         <f t="shared" si="8"/>
         <v>55.22</v>
       </c>
       <c r="F33">
-        <v>500</v>
+        <v>144</v>
       </c>
       <c r="G33">
         <f t="shared" si="9"/>
-        <v>5.8946034045635641E-3</v>
+        <v>6.1303875407461078E-3</v>
       </c>
       <c r="H33">
         <v>365</v>
       </c>
       <c r="I33">
         <f t="shared" si="10"/>
-        <v>1075.7651213328504</v>
+        <v>322.21316914161542</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>37</v>
       </c>
-      <c r="D34">
-        <f>$Q$13</f>
-        <v>1.71</v>
+      <c r="C34" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="D34" s="2">
+        <v>1.8</v>
       </c>
       <c r="E34">
         <f t="shared" si="8"/>
         <v>55.22</v>
       </c>
       <c r="F34">
-        <v>900</v>
+        <v>855</v>
       </c>
       <c r="G34">
         <f t="shared" si="9"/>
-        <v>4.031908728721478E-3</v>
+        <v>4.2441144512857668E-3</v>
       </c>
       <c r="H34">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="I34">
         <f t="shared" si="10"/>
-        <v>798.31792828685263</v>
+        <v>762.03074972835941</v>
       </c>
     </row>
   </sheetData>

</xml_diff>